<commit_message>
Update README and fix exception screenshot path
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stelligence365-my.sharepoint.com/personal/dawin_j_stelligence_com/Documents/Documents/UiPath/UiPath_Web_UI_Automation/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35F15BA4-17DB-45D3-BA84-7F6DCFC6F490}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B5FFF17-147C-41ED-80D6-01B5B8001389}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="59">
   <si>
     <t>Name</t>
   </si>
@@ -165,9 +165,6 @@
     <t>Data\Input\Input_Mockup_Data.xlsx</t>
   </si>
   <si>
-    <t>Input Folder</t>
-  </si>
-  <si>
     <t>URL</t>
   </si>
   <si>
@@ -199,6 +196,12 @@
   </si>
   <si>
     <t>Data\Output\Output_Report.xlsx</t>
+  </si>
+  <si>
+    <t>screenshots_folder</t>
+  </si>
+  <si>
+    <t>File Path</t>
   </si>
 </sst>
 </file>
@@ -588,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z1000"/>
+  <dimension ref="A1:Z1001"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -667,14 +670,14 @@
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" s="5" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
         <v>45</v>
@@ -682,57 +685,64 @@
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
         <v>56</v>
-      </c>
-      <c r="B10" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A13" s="5" t="s">
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" s="2"/>
+    </row>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A14" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+    </row>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
     </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A17" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-    </row>
+    <row r="17" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>52</v>
-      </c>
+      <c r="A18" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5"/>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>55</v>
-      </c>
     </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
@@ -1713,6 +1723,7 @@
     <row r="998" ht="14.25" customHeight="1"/>
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="1001" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>